<commit_message>
Revised 20260812 with updated pressure correction
</commit_message>
<xml_diff>
--- a/processing26/resultsTable_SHIP.xlsx
+++ b/processing26/resultsTable_SHIP.xlsx
@@ -1,6 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fileVersion appName="libxl" rupBuild="4.6.0"/>
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -13,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1585" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="4625" uniqueCount="63">
   <si>
     <t>fname</t>
   </si>
@@ -154,6 +155,54 @@
   </si>
   <si>
     <t>467</t>
+  </si>
+  <si>
+    <t>20260624_arr.c10.nc</t>
+  </si>
+  <si>
+    <t>552</t>
+  </si>
+  <si>
+    <t>389</t>
+  </si>
+  <si>
+    <t>20260626_arr.c10.nc</t>
+  </si>
+  <si>
+    <t>553</t>
+  </si>
+  <si>
+    <t>390</t>
+  </si>
+  <si>
+    <t>464</t>
+  </si>
+  <si>
+    <t>555</t>
+  </si>
+  <si>
+    <t>392</t>
+  </si>
+  <si>
+    <t>391</t>
+  </si>
+  <si>
+    <t>594</t>
+  </si>
+  <si>
+    <t>461</t>
+  </si>
+  <si>
+    <t>551</t>
+  </si>
+  <si>
+    <t>388</t>
+  </si>
+  <si>
+    <t>593</t>
+  </si>
+  <si>
+    <t>460</t>
   </si>
 </sst>
 </file>
@@ -199,35 +248,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z15"/>
+  <dimension ref="A1:Z24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="true"/>
+    <col min="1" max="1" width="19.7109375" customWidth="true"/>
     <col min="2" max="2" width="8.85546875" customWidth="true"/>
-    <col min="3" max="3" width="14.7109375" customWidth="true"/>
-    <col min="4" max="4" width="14.7109375" customWidth="true"/>
+    <col min="3" max="3" width="15.42578125" customWidth="true"/>
+    <col min="4" max="4" width="15.7109375" customWidth="true"/>
     <col min="5" max="5" width="14.7109375" customWidth="true"/>
-    <col min="6" max="6" width="16.42578125" customWidth="true"/>
+    <col min="6" max="6" width="15.7109375" customWidth="true"/>
     <col min="7" max="7" width="16.42578125" customWidth="true"/>
     <col min="8" max="8" width="16.42578125" customWidth="true"/>
     <col min="9" max="9" width="16.42578125" customWidth="true"/>
     <col min="10" max="10" width="16.42578125" customWidth="true"/>
     <col min="11" max="11" width="16.42578125" customWidth="true"/>
     <col min="12" max="12" width="12.7109375" customWidth="true"/>
-    <col min="13" max="13" width="12.7109375" customWidth="true"/>
-    <col min="14" max="14" width="12.7109375" customWidth="true"/>
-    <col min="15" max="15" width="15.42578125" customWidth="true"/>
+    <col min="13" max="13" width="13.7109375" customWidth="true"/>
+    <col min="14" max="14" width="13.7109375" customWidth="true"/>
+    <col min="15" max="15" width="16.42578125" customWidth="true"/>
     <col min="16" max="16" width="15.42578125" customWidth="true"/>
-    <col min="17" max="17" width="15.7109375" customWidth="true"/>
-    <col min="18" max="18" width="13.7109375" customWidth="true"/>
-    <col min="19" max="19" width="13.7109375" customWidth="true"/>
-    <col min="20" max="20" width="13.7109375" customWidth="true"/>
-    <col min="21" max="21" width="16.42578125" customWidth="true"/>
-    <col min="22" max="22" width="14.7109375" customWidth="true"/>
+    <col min="17" max="17" width="15.42578125" customWidth="true"/>
+    <col min="18" max="18" width="12.7109375" customWidth="true"/>
+    <col min="19" max="19" width="12.7109375" customWidth="true"/>
+    <col min="20" max="20" width="12.7109375" customWidth="true"/>
+    <col min="21" max="21" width="15.7109375" customWidth="true"/>
+    <col min="22" max="22" width="15.7109375" customWidth="true"/>
     <col min="23" max="23" width="14.7109375" customWidth="true"/>
-    <col min="24" max="24" width="12.42578125" customWidth="true"/>
-    <col min="25" max="25" width="13.42578125" customWidth="true"/>
-    <col min="26" max="26" width="13.42578125" customWidth="true"/>
+    <col min="24" max="24" width="14.42578125" customWidth="true"/>
+    <col min="25" max="25" width="14.42578125" customWidth="true"/>
+    <col min="26" max="26" width="14.42578125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -312,1006 +361,1708 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C2" s="0">
-        <v>0.013948657427951604</v>
+        <v>0.013796148848991607</v>
       </c>
       <c r="D2" s="0">
-        <v>0.017453292499609536</v>
+        <v>0.017453292502978959</v>
       </c>
       <c r="E2" s="0">
-        <v>0.020957927571267469</v>
+        <v>0.021110436156966311</v>
       </c>
       <c r="F2" s="0">
-        <v>-0.002937886313870779</v>
+        <v>-0.0037102004329563265</v>
       </c>
       <c r="G2" s="0">
-        <v>-0.0026985599028262388</v>
+        <v>-0.0034611299605504342</v>
       </c>
       <c r="H2" s="0">
-        <v>-0.0024592334917816986</v>
+        <v>-0.0032120594881445419</v>
       </c>
       <c r="I2" s="0">
-        <v>-0.0022132046668036729</v>
+        <v>-0.0022282979875034858</v>
       </c>
       <c r="J2" s="0">
-        <v>-0.0019766542948771726</v>
+        <v>-0.0019821042137898211</v>
       </c>
       <c r="K2" s="0">
-        <v>-0.0017401039229506721</v>
+        <v>-0.0017359104400761565</v>
       </c>
       <c r="L2" s="0">
-        <v>0.77594639633752582</v>
+        <v>0.76641247531415146</v>
       </c>
       <c r="M2" s="0">
-        <v>0.78175133532792263</v>
+        <v>0.77237965826706434</v>
       </c>
       <c r="N2" s="0">
-        <v>0.78755627431831943</v>
+        <v>0.77834684121997722</v>
       </c>
       <c r="O2" s="0">
-        <v>-0.02632552834749775</v>
+        <v>-0.028393229403472275</v>
       </c>
       <c r="P2" s="0">
-        <v>-0.025608895073956833</v>
+        <v>-0.027644601995395049</v>
       </c>
       <c r="Q2" s="0">
-        <v>-0.024892261800415917</v>
+        <v>-0.026895974587317823</v>
       </c>
       <c r="R2" s="0">
-        <v>0.79889966504245724</v>
+        <v>0.77364200633468794</v>
       </c>
       <c r="S2" s="0">
-        <v>0.81238248072608554</v>
+        <v>0.78746537500178015</v>
       </c>
       <c r="T2" s="0">
-        <v>0.82586529640971384</v>
+        <v>0.80128874366887237</v>
       </c>
       <c r="U2" s="0">
-        <v>0.0032158874131785497</v>
+        <v>0.0027348992022662231</v>
       </c>
       <c r="V2" s="0">
-        <v>0.0037944263105793258</v>
+        <v>0.0033310384230048162</v>
       </c>
       <c r="W2" s="0">
-        <v>0.0043729652079801014</v>
+        <v>0.0039271776437434097</v>
       </c>
       <c r="X2" s="0">
-        <v>-5.0586332295676835</v>
+        <v>-0.73688281300293135</v>
       </c>
       <c r="Y2" s="0">
-        <v>-5.0447613541844589</v>
+        <v>-0.72128198500394469</v>
       </c>
       <c r="Z2" s="0">
-        <v>-5.0308894788012344</v>
+        <v>-0.70568115700495804</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="C3" s="0">
-        <v>0.013309613869268355</v>
+        <v>0.013471613638286029</v>
       </c>
       <c r="D3" s="0">
-        <v>0.017453292508344428</v>
+        <v>0.017453292519369598</v>
       </c>
       <c r="E3" s="0">
-        <v>0.021596971147420499</v>
+        <v>0.021434971400453168</v>
       </c>
       <c r="F3" s="0">
-        <v>-0.0012859500781924609</v>
+        <v>-0.0013151529350747262</v>
       </c>
       <c r="G3" s="0">
-        <v>-0.0010153984761985151</v>
+        <v>-0.0010552797105670853</v>
       </c>
       <c r="H3" s="0">
-        <v>-0.00074484687420456948</v>
+        <v>-0.00079540648605944445</v>
       </c>
       <c r="I3" s="0">
-        <v>-0.00063204872814472623</v>
+        <v>-0.00052240888763405678</v>
       </c>
       <c r="J3" s="0">
-        <v>-0.00036679992823318515</v>
+        <v>-0.00026763475663411657</v>
       </c>
       <c r="K3" s="0">
-        <v>-0.00010155112832164407</v>
+        <v>-1.2860625634176365e-05</v>
       </c>
       <c r="L3" s="0">
-        <v>0.77403660364455318</v>
+        <v>0.76151732289495566</v>
       </c>
       <c r="M3" s="0">
-        <v>0.78080740231115497</v>
+        <v>0.76791062309293812</v>
       </c>
       <c r="N3" s="0">
-        <v>0.78757820097775677</v>
+        <v>0.77430392329092057</v>
       </c>
       <c r="O3" s="0">
-        <v>-0.024098353661426746</v>
+        <v>-0.024391685354071595</v>
       </c>
       <c r="P3" s="0">
-        <v>-0.023290048305809094</v>
+        <v>-0.023613754741642085</v>
       </c>
       <c r="Q3" s="0">
-        <v>-0.022481742950191442</v>
+        <v>-0.022835824129212576</v>
       </c>
       <c r="R3" s="0">
-        <v>0.70801822472161013</v>
+        <v>0.69676925251800226</v>
       </c>
       <c r="S3" s="0">
-        <v>0.7226788561580435</v>
+        <v>0.71064813462452581</v>
       </c>
       <c r="T3" s="0">
-        <v>0.73733948759447687</v>
+        <v>0.72452701673104936</v>
       </c>
       <c r="U3" s="0">
-        <v>0.0028606109457724807</v>
+        <v>0.0027277059651523387</v>
       </c>
       <c r="V3" s="0">
-        <v>0.0035199279787753771</v>
+        <v>0.0033605797579225657</v>
       </c>
       <c r="W3" s="0">
-        <v>0.0041792450117782735</v>
+        <v>0.0039934535506927927</v>
       </c>
       <c r="X3" s="0">
-        <v>-5.0038083718310569</v>
+        <v>-0.45375562132209091</v>
       </c>
       <c r="Y3" s="0">
-        <v>-4.9877606897787459</v>
+        <v>-0.43738127592719483</v>
       </c>
       <c r="Z3" s="0">
-        <v>-4.9717130077264349</v>
+        <v>-0.42100693053229876</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C4" s="0">
-        <v>0.0020384262988475555</v>
+        <v>0.0033789176186130214</v>
       </c>
       <c r="D4" s="0">
-        <v>0.0074225801067767088</v>
+        <v>0.0084731399021472607</v>
       </c>
       <c r="E4" s="0">
-        <v>0.012806733914705862</v>
+        <v>0.013567362185681501</v>
       </c>
       <c r="F4" s="0">
-        <v>0.016101168850975817</v>
+        <v>0.016159176819595184</v>
       </c>
       <c r="G4" s="0">
-        <v>0.017453292396844899</v>
+        <v>0.017453292477796267</v>
       </c>
       <c r="H4" s="0">
-        <v>0.018805415942713982</v>
+        <v>0.018747408135997349</v>
       </c>
       <c r="I4" s="0">
-        <v>0.022823649646153223</v>
+        <v>0.017387801339523504</v>
       </c>
       <c r="J4" s="0">
-        <v>0.028132462918619674</v>
+        <v>0.022539289649647031</v>
       </c>
       <c r="K4" s="0">
-        <v>0.033441276191086125</v>
+        <v>0.027690777959770558</v>
       </c>
       <c r="L4" s="0">
-        <v>0.4391231883963278</v>
+        <v>0.4572564282302416</v>
       </c>
       <c r="M4" s="0">
-        <v>0.5310416645178867</v>
+        <v>0.54509889441655623</v>
       </c>
       <c r="N4" s="0">
-        <v>0.6229601406394456</v>
+        <v>0.63294136060287087</v>
       </c>
       <c r="O4" s="0">
-        <v>0.025988826939071091</v>
+        <v>0.024188770747897874</v>
       </c>
       <c r="P4" s="0">
-        <v>0.03412047096963991</v>
+        <v>0.032089908843038535</v>
       </c>
       <c r="Q4" s="0">
-        <v>0.042252115000208729</v>
+        <v>0.039991046938179196</v>
       </c>
       <c r="R4" s="0">
-        <v>0.73370494903434946</v>
+        <v>0.72676880588190551</v>
       </c>
       <c r="S4" s="0">
-        <v>0.74414362558688052</v>
+        <v>0.73611451831627095</v>
       </c>
       <c r="T4" s="0">
-        <v>0.75458230213941158</v>
+        <v>0.74546023075063639</v>
       </c>
       <c r="U4" s="0">
-        <v>-0.00031081458619803756</v>
+        <v>0.00049681708166833235</v>
       </c>
       <c r="V4" s="0">
-        <v>0.0023350299198718534</v>
+        <v>0.0030491763661513989</v>
       </c>
       <c r="W4" s="0">
-        <v>0.0049808744259417443</v>
+        <v>0.0056015356506344659</v>
       </c>
       <c r="X4" s="0">
-        <v>-15.811108410896829</v>
+        <v>-11.520870913439333</v>
       </c>
       <c r="Y4" s="0">
-        <v>-14.387223433739205</v>
+        <v>-10.181827394116441</v>
       </c>
       <c r="Z4" s="0">
-        <v>-12.963338456581582</v>
+        <v>-8.8427838747935486</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="C5" s="0">
-        <v>-0.010010182531739169</v>
+        <v>-0.010923255052409184</v>
       </c>
       <c r="D5" s="0">
-        <v>0.0024574239044129103</v>
+        <v>0.0020760125369999388</v>
       </c>
       <c r="E5" s="0">
-        <v>0.014925030340564992</v>
+        <v>0.015075280126409064</v>
       </c>
       <c r="F5" s="0">
-        <v>0.013478033025195478</v>
+        <v>0.014221822232093182</v>
       </c>
       <c r="G5" s="0">
-        <v>0.016611986288103856</v>
+        <v>0.017453292395101832</v>
       </c>
       <c r="H5" s="0">
-        <v>0.019745939551012233</v>
+        <v>0.020684762558110484</v>
       </c>
       <c r="I5" s="0">
-        <v>-0.01684820417153499</v>
+        <v>-0.021513602891010855</v>
       </c>
       <c r="J5" s="0">
-        <v>-0.0062397161306523416</v>
+        <v>-0.010534755969131908</v>
       </c>
       <c r="K5" s="0">
-        <v>0.0043687719102303074</v>
+        <v>0.00044409095274703693</v>
       </c>
       <c r="L5" s="0">
-        <v>0.56138776085268405</v>
+        <v>0.50012679614525035</v>
       </c>
       <c r="M5" s="0">
-        <v>0.77444441278373577</v>
+        <v>0.71601033481974108</v>
       </c>
       <c r="N5" s="0">
-        <v>0.98750106471478749</v>
+        <v>0.93189387349423181</v>
       </c>
       <c r="O5" s="0">
-        <v>-0.0015716451308502109</v>
+        <v>0.002826923483536161</v>
       </c>
       <c r="P5" s="0">
-        <v>0.015316914253864703</v>
+        <v>0.020293064053763316</v>
       </c>
       <c r="Q5" s="0">
-        <v>0.032205473638579618</v>
+        <v>0.037759204623990475</v>
       </c>
       <c r="R5" s="0">
-        <v>0.65172048647254666</v>
+        <v>0.62979469040800495</v>
       </c>
       <c r="S5" s="0">
-        <v>0.66985107680334466</v>
+        <v>0.64826370881182449</v>
       </c>
       <c r="T5" s="0">
-        <v>0.68798166713414266</v>
+        <v>0.66673272721564403</v>
       </c>
       <c r="U5" s="0">
-        <v>-0.0031228722395326355</v>
+        <v>-0.0053753642063215073</v>
       </c>
       <c r="V5" s="0">
-        <v>0.0039339530002159943</v>
+        <v>0.0020217192593385723</v>
       </c>
       <c r="W5" s="0">
-        <v>0.010990778239964624</v>
+        <v>0.0094188027249986518</v>
       </c>
       <c r="X5" s="0">
-        <v>-10.681910422505348</v>
+        <v>-8.4735217400053848</v>
       </c>
       <c r="Y5" s="0">
-        <v>-8.323403116191022</v>
+        <v>-6.0344887499139137</v>
       </c>
       <c r="Z5" s="0">
-        <v>-5.9648958098766958</v>
+        <v>-3.5954557598224422</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C6" s="0">
-        <v>0.015387820649723239</v>
+        <v>0.015488725066334121</v>
       </c>
       <c r="D6" s="0">
-        <v>0.0174532925199078</v>
+        <v>0.017453292518585621</v>
       </c>
       <c r="E6" s="0">
-        <v>0.019518764390092362</v>
+        <v>0.019417859970837122</v>
       </c>
       <c r="F6" s="0">
-        <v>0.00036817955334520776</v>
+        <v>0.0001506671194881325</v>
       </c>
       <c r="G6" s="0">
-        <v>0.00050546420354583531</v>
+        <v>0.00028108066502495661</v>
       </c>
       <c r="H6" s="0">
-        <v>0.00064274885374646291</v>
+        <v>0.00041149421056178073</v>
       </c>
       <c r="I6" s="0">
-        <v>-0.00090592024694081995</v>
+        <v>-0.00080553616917807122</v>
       </c>
       <c r="J6" s="0">
-        <v>-0.00076878836048285587</v>
+        <v>-0.00067526844007368369</v>
       </c>
       <c r="K6" s="0">
-        <v>-0.00063165647402489179</v>
+        <v>-0.00054500071096929615</v>
       </c>
       <c r="L6" s="0">
-        <v>0.8449211988588653</v>
+        <v>0.83264030296755687</v>
       </c>
       <c r="M6" s="0">
-        <v>0.84928672435457897</v>
+        <v>0.83672439652871278</v>
       </c>
       <c r="N6" s="0">
-        <v>0.85365224985029264</v>
+        <v>0.84080849008986869</v>
       </c>
       <c r="O6" s="0">
-        <v>-0.020462962792295078</v>
+        <v>-0.021232489223868202</v>
       </c>
       <c r="P6" s="0">
-        <v>-0.019995863772198148</v>
+        <v>-0.020787395353420109</v>
       </c>
       <c r="Q6" s="0">
-        <v>-0.019528764752101219</v>
+        <v>-0.020342301482972017</v>
       </c>
       <c r="R6" s="0">
-        <v>0.78402768187700978</v>
+        <v>0.77043494062867024</v>
       </c>
       <c r="S6" s="0">
-        <v>0.78923741827754135</v>
+        <v>0.77531522432552835</v>
       </c>
       <c r="T6" s="0">
-        <v>0.79444715467807292</v>
+        <v>0.78019550802238646</v>
       </c>
       <c r="U6" s="0">
-        <v>0.0047933997213672934</v>
+        <v>0.0045957430917924844</v>
       </c>
       <c r="V6" s="0">
-        <v>0.0051518154585214861</v>
+        <v>0.0049352569192693098</v>
       </c>
       <c r="W6" s="0">
-        <v>0.0055102311956756788</v>
+        <v>0.0052747707467461352</v>
       </c>
       <c r="X6" s="0">
-        <v>-4.913250030240941</v>
+        <v>-0.75174176828181683</v>
       </c>
       <c r="Y6" s="0">
-        <v>-4.9047840239160809</v>
+        <v>-0.74304790164608847</v>
       </c>
       <c r="Z6" s="0">
-        <v>-4.8963180175912209</v>
+        <v>-0.73435403501036012</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C7" s="0">
-        <v>0.006184681904769453</v>
+        <v>-0.0036883022907283078</v>
       </c>
       <c r="D7" s="0">
-        <v>0.010219114202352563</v>
+        <v>0.00092386585576805468</v>
       </c>
       <c r="E7" s="0">
-        <v>0.014253546499935673</v>
+        <v>0.0055360340022644174</v>
       </c>
       <c r="F7" s="0">
-        <v>0.0019770698138932286</v>
+        <v>0.0039214030032957026</v>
       </c>
       <c r="G7" s="0">
-        <v>0.0033061030674676533</v>
+        <v>0.0051046165257119733</v>
       </c>
       <c r="H7" s="0">
-        <v>0.0046351363210420781</v>
+        <v>0.0062878300481282439</v>
       </c>
       <c r="I7" s="0">
-        <v>0.0089131023907188488</v>
+        <v>0.00062982242928778798</v>
       </c>
       <c r="J7" s="0">
-        <v>0.012441466268947684</v>
+        <v>0.0048220727102142565</v>
       </c>
       <c r="K7" s="0">
-        <v>0.015969830147176518</v>
+        <v>0.009014322991140725</v>
       </c>
       <c r="L7" s="0">
-        <v>0.65083966949436622</v>
+        <v>0.70389404058719574</v>
       </c>
       <c r="M7" s="0">
-        <v>0.73057635736752402</v>
+        <v>0.80069108504127218</v>
       </c>
       <c r="N7" s="0">
-        <v>0.81031304524068182</v>
+        <v>0.89748812949534862</v>
       </c>
       <c r="O7" s="0">
-        <v>-0.019223641523590174</v>
+        <v>-0.019466059688426247</v>
       </c>
       <c r="P7" s="0">
-        <v>-0.013226735183276247</v>
+        <v>-0.012283411447464806</v>
       </c>
       <c r="Q7" s="0">
-        <v>-0.0072298288429623178</v>
+        <v>-0.005100763206503366</v>
       </c>
       <c r="R7" s="0">
-        <v>0.79531077835874875</v>
+        <v>0.78008203032057777</v>
       </c>
       <c r="S7" s="0">
-        <v>0.80180948284600007</v>
+        <v>0.78797220646588495</v>
       </c>
       <c r="T7" s="0">
-        <v>0.80830818733325138</v>
+        <v>0.79586238261119213</v>
       </c>
       <c r="U7" s="0">
-        <v>0.0091793300134002595</v>
+        <v>0.0015025361071070915</v>
       </c>
       <c r="V7" s="0">
-        <v>0.012095922900977359</v>
+        <v>0.0038234430987622537</v>
       </c>
       <c r="W7" s="0">
-        <v>0.015012515788554458</v>
+        <v>0.0061443500904174164</v>
       </c>
       <c r="X7" s="0">
-        <v>-1.4353552246128529</v>
+        <v>6.5667345952727532</v>
       </c>
       <c r="Y7" s="0">
-        <v>-0.7599836000559973</v>
+        <v>7.9858164417800808</v>
       </c>
       <c r="Z7" s="0">
-        <v>-0.084611975499141678</v>
+        <v>9.4048982882874075</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="0"/>
-      <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
-      <c r="E8" s="0"/>
-      <c r="F8" s="0"/>
-      <c r="G8" s="0"/>
-      <c r="H8" s="0"/>
-      <c r="I8" s="0"/>
-      <c r="J8" s="0"/>
-      <c r="K8" s="0"/>
-      <c r="L8" s="0"/>
-      <c r="M8" s="0"/>
-      <c r="N8" s="0"/>
-      <c r="O8" s="0"/>
-      <c r="P8" s="0"/>
-      <c r="Q8" s="0"/>
-      <c r="R8" s="0"/>
-      <c r="S8" s="0"/>
-      <c r="T8" s="0"/>
-      <c r="U8" s="0"/>
-      <c r="V8" s="0"/>
-      <c r="W8" s="0"/>
-      <c r="X8" s="0"/>
-      <c r="Y8" s="0"/>
-      <c r="Z8" s="0"/>
+      <c r="A8" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="0">
+        <v>0.0067423814184362982</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0.010885850102746248</v>
+      </c>
+      <c r="E8" s="0">
+        <v>0.015029318787056198</v>
+      </c>
+      <c r="F8" s="0">
+        <v>0.0024362034208628503</v>
+      </c>
+      <c r="G8" s="0">
+        <v>0.0037926595520403647</v>
+      </c>
+      <c r="H8" s="0">
+        <v>0.0051491156832178791</v>
+      </c>
+      <c r="I8" s="0">
+        <v>0.0049184844056796677</v>
+      </c>
+      <c r="J8" s="0">
+        <v>0.0085475114728210608</v>
+      </c>
+      <c r="K8" s="0">
+        <v>0.012176538539962454</v>
+      </c>
+      <c r="L8" s="0">
+        <v>0.60314907653626426</v>
+      </c>
+      <c r="M8" s="0">
+        <v>0.68300634352365131</v>
+      </c>
+      <c r="N8" s="0">
+        <v>0.76286361051103835</v>
+      </c>
+      <c r="O8" s="0">
+        <v>-0.016211354299034978</v>
+      </c>
+      <c r="P8" s="0">
+        <v>-0.01007860741944072</v>
+      </c>
+      <c r="Q8" s="0">
+        <v>-0.0039458605398464608</v>
+      </c>
+      <c r="R8" s="0">
+        <v>0.77978262043677482</v>
+      </c>
+      <c r="S8" s="0">
+        <v>0.78630232255653532</v>
+      </c>
+      <c r="T8" s="0">
+        <v>0.79282202467629581</v>
+      </c>
+      <c r="U8" s="0">
+        <v>0.0084959625748527289</v>
+      </c>
+      <c r="V8" s="0">
+        <v>0.011481102745694249</v>
+      </c>
+      <c r="W8" s="0">
+        <v>0.01446624291653577</v>
+      </c>
+      <c r="X8" s="0">
+        <v>1.885667288071228</v>
+      </c>
+      <c r="Y8" s="0">
+        <v>2.6356551618877724</v>
+      </c>
+      <c r="Z8" s="0">
+        <v>3.3856430357043168</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="0"/>
+        <v>47</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>54</v>
+      </c>
       <c r="C9" s="0">
-        <v>0.0068098362698035056</v>
+        <v>0.0010272278156979015</v>
       </c>
       <c r="D9" s="0">
-        <v>0.012076499290233992</v>
+        <v>0.0041583967243602107</v>
       </c>
       <c r="E9" s="0">
-        <v>0.017343162310664472</v>
+        <v>0.0072895656330225194</v>
       </c>
       <c r="F9" s="0">
-        <v>0.004616769141891082</v>
+        <v>-0.0040295137568664968</v>
       </c>
       <c r="G9" s="0">
-        <v>0.0056938145961562487</v>
+        <v>-0.0038536124723047181</v>
       </c>
       <c r="H9" s="0">
-        <v>0.0067708600504214145</v>
+        <v>-0.0036777111877429394</v>
       </c>
       <c r="I9" s="0">
-        <v>0.0018562290372413106</v>
+        <v>-0.00079111116013829926</v>
       </c>
       <c r="J9" s="0">
-        <v>0.0052036617455536336</v>
+        <v>-0.00061082504668464601</v>
       </c>
       <c r="K9" s="0">
-        <v>0.0085510944538659574</v>
+        <v>-0.00043053893323099276</v>
       </c>
       <c r="L9" s="0">
-        <v>0.67437580293072041</v>
+        <v>0.69231914045656351</v>
       </c>
       <c r="M9" s="0">
-        <v>0.7413179827771339</v>
+        <v>0.71437198331333263</v>
       </c>
       <c r="N9" s="0">
-        <v>0.80826016262354727</v>
+        <v>0.73642482617010174</v>
       </c>
       <c r="O9" s="0">
-        <v>-0.010948884086098143</v>
+        <v>-0.026218130294046151</v>
       </c>
       <c r="P9" s="0">
-        <v>-0.0054473595186226185</v>
+        <v>-0.02396976280794343</v>
       </c>
       <c r="Q9" s="0">
-        <v>5.4165048852908671e-05</v>
+        <v>-0.021721395321840708</v>
       </c>
       <c r="R9" s="0">
-        <v>0.74528029758445369</v>
+        <v>0.77447741555454253</v>
       </c>
       <c r="S9" s="0">
-        <v>0.75668382339964924</v>
+        <v>0.77926312591219216</v>
       </c>
       <c r="T9" s="0">
-        <v>0.76808734921484501</v>
+        <v>0.78404883626984179</v>
       </c>
       <c r="U9" s="0">
-        <v>0.002769256877997985</v>
+        <v>0.0072495590400039264</v>
       </c>
       <c r="V9" s="0">
-        <v>0.0051385125948235659</v>
+        <v>0.007721571079848848</v>
       </c>
       <c r="W9" s="0">
-        <v>0.0075077683116491463</v>
+        <v>0.0081935831196937696</v>
       </c>
       <c r="X9" s="0">
-        <v>-7.1506776149424516</v>
+        <v>-0.31072595246624729</v>
       </c>
       <c r="Y9" s="0">
-        <v>-6.4013193696442512</v>
+        <v>-0.29717081819581048</v>
       </c>
       <c r="Z9" s="0">
-        <v>-5.6519611243460517</v>
+        <v>-0.28361568392537367</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="0"/>
+        <v>47</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>54</v>
+      </c>
       <c r="C10" s="0">
-        <v>0.0097248331190615614</v>
+        <v>0.013091287876697274</v>
       </c>
       <c r="D10" s="0">
-        <v>0.0063932021768487255</v>
+        <v>0.01533660770618357</v>
       </c>
       <c r="E10" s="0">
-        <v>0.00379122493638452</v>
+        <v>0.017581927535669867</v>
       </c>
       <c r="F10" s="0">
-        <v>0.0080913147703958379</v>
+        <v>0.00039605053593986546</v>
       </c>
       <c r="G10" s="0">
-        <v>0.0090061915054244317</v>
+        <v>0.00050946661500639128</v>
       </c>
       <c r="H10" s="0">
-        <v>0.0099697418585749081</v>
+        <v>0.00062288269407291715</v>
       </c>
       <c r="I10" s="0">
-        <v>0.013188398657585832</v>
+        <v>0.00052831487452158828</v>
       </c>
       <c r="J10" s="0">
-        <v>0.012863310435025577</v>
+        <v>0.00064017647079376184</v>
       </c>
       <c r="K10" s="0">
-        <v>0.013835827132944931</v>
+        <v>0.00075203806706593539</v>
       </c>
       <c r="L10" s="0">
-        <v>0.15362202484751336</v>
+        <v>0.7398213710030066</v>
       </c>
       <c r="M10" s="0">
-        <v>0.10980017514879864</v>
+        <v>0.74337825860198059</v>
       </c>
       <c r="N10" s="0">
-        <v>0.11780021185728286</v>
+        <v>0.74693514620095458</v>
       </c>
       <c r="O10" s="0">
-        <v>0.02010306518585608</v>
+        <v>-0.017607494169486558</v>
       </c>
       <c r="P10" s="0">
-        <v>0.024469552491617776</v>
+        <v>-0.017122200596019068</v>
       </c>
       <c r="Q10" s="0">
-        <v>0.029601056375140988</v>
+        <v>-0.016636907022551578</v>
       </c>
       <c r="R10" s="0">
-        <v>0.058575309450324763</v>
+        <v>0.77620673278297625</v>
       </c>
       <c r="S10" s="0">
-        <v>0.054866970661143349</v>
+        <v>0.78226757012630011</v>
       </c>
       <c r="T10" s="0">
-        <v>0.051372334845535023</v>
+        <v>0.78832840746962396</v>
       </c>
       <c r="U10" s="0">
-        <v>0.0042331558443891616</v>
+        <v>0.0061781320130268862</v>
       </c>
       <c r="V10" s="0">
-        <v>0.0035254105621579592</v>
+        <v>0.0066009561898845194</v>
       </c>
       <c r="W10" s="0">
-        <v>0.0044661840076005432</v>
+        <v>0.0070237803667421526</v>
       </c>
       <c r="X10" s="0">
-        <v>5.1793697723237591</v>
+        <v>-0.042785915856796662</v>
       </c>
       <c r="Y10" s="0">
-        <v>4.5906808807985886</v>
+        <v>-0.03695832521044834</v>
       </c>
       <c r="Z10" s="0">
-        <v>4.1465408993702804</v>
+        <v>-0.03113073456410002</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="0"/>
-      <c r="B11" s="0"/>
-      <c r="C11" s="0"/>
-      <c r="D11" s="0"/>
-      <c r="E11" s="0"/>
-      <c r="F11" s="0"/>
-      <c r="G11" s="0"/>
-      <c r="H11" s="0"/>
-      <c r="I11" s="0"/>
-      <c r="J11" s="0"/>
-      <c r="K11" s="0"/>
-      <c r="L11" s="0"/>
-      <c r="M11" s="0"/>
-      <c r="N11" s="0"/>
-      <c r="O11" s="0"/>
-      <c r="P11" s="0"/>
-      <c r="Q11" s="0"/>
-      <c r="R11" s="0"/>
-      <c r="S11" s="0"/>
-      <c r="T11" s="0"/>
-      <c r="U11" s="0"/>
-      <c r="V11" s="0"/>
-      <c r="W11" s="0"/>
-      <c r="X11" s="0"/>
-      <c r="Y11" s="0"/>
-      <c r="Z11" s="0"/>
+      <c r="A11" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="0">
+        <v>-0.0010195216857747909</v>
+      </c>
+      <c r="D11" s="0">
+        <v>0.0043750838059252598</v>
+      </c>
+      <c r="E11" s="0">
+        <v>0.0097696892976253114</v>
+      </c>
+      <c r="F11" s="0">
+        <v>0.0013962174191912932</v>
+      </c>
+      <c r="G11" s="0">
+        <v>0.003855096591234597</v>
+      </c>
+      <c r="H11" s="0">
+        <v>0.0063139757632779004</v>
+      </c>
+      <c r="I11" s="0">
+        <v>-0.04237299684731994</v>
+      </c>
+      <c r="J11" s="0">
+        <v>-0.034906582811064374</v>
+      </c>
+      <c r="K11" s="0">
+        <v>-0.027440168774808808</v>
+      </c>
+      <c r="L11" s="0">
+        <v>0.64137178270156281</v>
+      </c>
+      <c r="M11" s="0">
+        <v>0.70745813062978902</v>
+      </c>
+      <c r="N11" s="0">
+        <v>0.77354447855801523</v>
+      </c>
+      <c r="O11" s="0">
+        <v>-0.013193292182913485</v>
+      </c>
+      <c r="P11" s="0">
+        <v>-0.0058628365542440636</v>
+      </c>
+      <c r="Q11" s="0">
+        <v>0.0014676190744253581</v>
+      </c>
+      <c r="R11" s="0">
+        <v>0.76868720017837067</v>
+      </c>
+      <c r="S11" s="0">
+        <v>0.77684449305774583</v>
+      </c>
+      <c r="T11" s="0">
+        <v>0.785001785937121</v>
+      </c>
+      <c r="U11" s="0">
+        <v>-0.0042874724337891735</v>
+      </c>
+      <c r="V11" s="0">
+        <v>0.00098673745819003985</v>
+      </c>
+      <c r="W11" s="0">
+        <v>0.0062609473501692541</v>
+      </c>
+      <c r="X11" s="0">
+        <v>2.5251110061638506</v>
+      </c>
+      <c r="Y11" s="0">
+        <v>3.972782877571198</v>
+      </c>
+      <c r="Z11" s="0">
+        <v>5.4204547489785453</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="0"/>
+        <v>50</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>53</v>
+      </c>
       <c r="C12" s="0">
-        <v>0.015678641248588466</v>
+        <v>0.013711400381021288</v>
       </c>
       <c r="D12" s="0">
-        <v>0.017453292519911963</v>
+        <v>0.017453219229896177</v>
       </c>
       <c r="E12" s="0">
-        <v>0.01922794379123546</v>
+        <v>0.021195038078771066</v>
       </c>
       <c r="F12" s="0">
-        <v>-0.00095379816614962092</v>
+        <v>0.0044336680251024288</v>
       </c>
       <c r="G12" s="0">
-        <v>-0.00083166635979889175</v>
+        <v>0.0046725439003982528</v>
       </c>
       <c r="H12" s="0">
-        <v>-0.00070953455344816257</v>
+        <v>0.0049114197756940769</v>
       </c>
       <c r="I12" s="0">
-        <v>-0.0015401257001548708</v>
+        <v>0.0014254027485168666</v>
       </c>
       <c r="J12" s="0">
-        <v>-0.0014181212713143814</v>
+        <v>0.0016674587423236276</v>
       </c>
       <c r="K12" s="0">
-        <v>-0.001296116842473892</v>
+        <v>0.0019095147361303886</v>
       </c>
       <c r="L12" s="0">
-        <v>0.79519359114799637</v>
+        <v>0.84042749564163854</v>
       </c>
       <c r="M12" s="0">
-        <v>0.79844785803642393</v>
+        <v>0.86002224227047186</v>
       </c>
       <c r="N12" s="0">
-        <v>0.80170212492485149</v>
+        <v>0.87961698889930518</v>
       </c>
       <c r="O12" s="0">
-        <v>-0.022457342141524818</v>
+        <v>-0.021768978443207986</v>
       </c>
       <c r="P12" s="0">
-        <v>-0.022079838041080682</v>
+        <v>-0.019661809766329672</v>
       </c>
       <c r="Q12" s="0">
-        <v>-0.021702333940636545</v>
+        <v>-0.017554641089451359</v>
       </c>
       <c r="R12" s="0">
-        <v>0.78152012534727611</v>
+        <v>0.76078214752986406</v>
       </c>
       <c r="S12" s="0">
-        <v>0.78641411575112141</v>
+        <v>0.76677801824794611</v>
       </c>
       <c r="T12" s="0">
-        <v>0.79130810615496672</v>
+        <v>0.77277388896602817</v>
       </c>
       <c r="U12" s="0">
-        <v>0.0045285711494369042</v>
+        <v>0.0046146088440916595</v>
       </c>
       <c r="V12" s="0">
-        <v>0.004832689517453745</v>
+        <v>0.0053655283253346555</v>
       </c>
       <c r="W12" s="0">
-        <v>0.0051368078854705859</v>
+        <v>0.0061164478065776516</v>
       </c>
       <c r="X12" s="0">
-        <v>-4.9861707886482494</v>
+        <v>-0.35747011018888314</v>
       </c>
       <c r="Y12" s="0">
-        <v>-4.9787612205420917</v>
+        <v>-0.3398236245130154</v>
       </c>
       <c r="Z12" s="0">
-        <v>-4.971351652435934</v>
+        <v>-0.32217713883714766</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" s="0"/>
+        <v>50</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>53</v>
+      </c>
       <c r="C13" s="0">
-        <v>0.0081191475840305064</v>
+        <v>0.0010705153513174909</v>
       </c>
       <c r="D13" s="0">
-        <v>0.012042443303155403</v>
+        <v>0.0059280148711249713</v>
       </c>
       <c r="E13" s="0">
-        <v>0.01604681165580792</v>
+        <v>0.010785514390932453</v>
       </c>
       <c r="F13" s="0">
-        <v>0.004383877844164866</v>
+        <v>0.0018580401057492753</v>
       </c>
       <c r="G13" s="0">
-        <v>0.0053368030354132533</v>
+        <v>0.0020836308876135156</v>
       </c>
       <c r="H13" s="0">
-        <v>0.0062951364064529614</v>
+        <v>0.002309221669477756</v>
       </c>
       <c r="I13" s="0">
-        <v>0.0027379862464577925</v>
+        <v>0.0011098943575592666</v>
       </c>
       <c r="J13" s="0">
-        <v>0.005318980153620736</v>
+        <v>0.0013291485771579352</v>
       </c>
       <c r="K13" s="0">
-        <v>0.008044152385281415</v>
+        <v>0.0015484027967566038</v>
       </c>
       <c r="L13" s="0">
-        <v>0.62993847072339482</v>
+        <v>0.84877983526052825</v>
       </c>
       <c r="M13" s="0">
-        <v>0.67749710140279551</v>
+        <v>0.85615888642614568</v>
       </c>
       <c r="N13" s="0">
-        <v>0.73081371946077389</v>
+        <v>0.86353793759176312</v>
       </c>
       <c r="O13" s="0">
-        <v>-0.0087773850620395267</v>
+        <v>-0.027387740724083218</v>
       </c>
       <c r="P13" s="0">
-        <v>-0.0039713113533134704</v>
+        <v>-0.026355107390931654</v>
       </c>
       <c r="Q13" s="0">
-        <v>0.00091976419738608935</v>
+        <v>-0.025322474057780091</v>
       </c>
       <c r="R13" s="0">
-        <v>0.67300639087653069</v>
+        <v>0.73170173774468394</v>
       </c>
       <c r="S13" s="0">
-        <v>0.68200753891220112</v>
+        <v>0.7475882997265797</v>
       </c>
       <c r="T13" s="0">
-        <v>0.691032431722713</v>
+        <v>0.76347486170847545</v>
       </c>
       <c r="U13" s="0">
-        <v>0.0031273916822013286</v>
+        <v>0.00051957359693336695</v>
       </c>
       <c r="V13" s="0">
-        <v>0.0049252986937085184</v>
+        <v>0.0014755085276827408</v>
       </c>
       <c r="W13" s="0">
-        <v>0.0069063744527350177</v>
+        <v>0.0024314434584321145</v>
       </c>
       <c r="X13" s="0">
-        <v>-5.5401715912135172</v>
+        <v>-0.13658723435922737</v>
       </c>
       <c r="Y13" s="0">
-        <v>-5.0219239919170287</v>
+        <v>-0.12411931797857205</v>
       </c>
       <c r="Z13" s="0">
-        <v>-4.4876154026097801</v>
+        <v>-0.11165140159791673</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" s="0"/>
+        <v>50</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>53</v>
+      </c>
       <c r="C14" s="0">
-        <v>0.0082506525445932375</v>
+        <v>0.0094037815957136763</v>
       </c>
       <c r="D14" s="0">
-        <v>0.0057615590727655647</v>
+        <v>0.017453292511261598</v>
       </c>
       <c r="E14" s="0">
-        <v>0.0055221102763584095</v>
+        <v>0.025502803426809519</v>
       </c>
       <c r="F14" s="0">
-        <v>0.006800389840085394</v>
+        <v>0.0080454930148425446</v>
       </c>
       <c r="G14" s="0">
-        <v>0.0075660760500981033</v>
+        <v>0.0092716172182242367</v>
       </c>
       <c r="H14" s="0">
-        <v>0.008375045485073231</v>
+        <v>0.010497741421605929</v>
       </c>
       <c r="I14" s="0">
-        <v>0.011195005178535562</v>
+        <v>-0.0019309891363610068</v>
       </c>
       <c r="J14" s="0">
-        <v>0.010780319569072664</v>
+        <v>-0.00071929598988773093</v>
       </c>
       <c r="K14" s="0">
-        <v>0.011617517052492633</v>
+        <v>0.00049239715658554487</v>
       </c>
       <c r="L14" s="0">
-        <v>0.21966109677340473</v>
+        <v>0.72355645056385498</v>
       </c>
       <c r="M14" s="0">
-        <v>0.23067862173861034</v>
+        <v>0.73677601153753103</v>
       </c>
       <c r="N14" s="0">
-        <v>0.24803750649136494</v>
+        <v>0.74999557251120708</v>
       </c>
       <c r="O14" s="0">
-        <v>0.019605151228797111</v>
+        <v>-0.00036911263280190029</v>
       </c>
       <c r="P14" s="0">
-        <v>0.022764686188403386</v>
+        <v>0.0024434088381772843</v>
       </c>
       <c r="Q14" s="0">
-        <v>0.026741198016765805</v>
+        <v>0.0052559303091564685</v>
       </c>
       <c r="R14" s="0">
-        <v>0.2353244414402034</v>
+        <v>0.93706000171390469</v>
       </c>
       <c r="S14" s="0">
-        <v>0.23934644875031227</v>
+        <v>0.97111492772343766</v>
       </c>
       <c r="T14" s="0">
-        <v>0.24340759451104019</v>
+        <v>1.0051698537329707</v>
       </c>
       <c r="U14" s="0">
-        <v>0.0034220221372399913</v>
+        <v>0.0085620751209391187</v>
       </c>
       <c r="V14" s="0">
-        <v>0.0028378927607614528</v>
+        <v>0.011157280617098997</v>
       </c>
       <c r="W14" s="0">
-        <v>0.0037308111585822932</v>
+        <v>0.013752486113258876</v>
       </c>
       <c r="X14" s="0">
-        <v>5.7825269961908221</v>
+        <v>0.30143529740722363</v>
       </c>
       <c r="Y14" s="0">
-        <v>5.136814570664197</v>
+        <v>0.34457879128216779</v>
       </c>
       <c r="Z14" s="0">
-        <v>4.6130463047108208</v>
+        <v>0.38772228515711194</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="0">
+        <v>0.0019717609762513778</v>
+      </c>
+      <c r="D15" s="0">
+        <v>0.0061443380700334097</v>
+      </c>
+      <c r="E15" s="0">
+        <v>0.010316915163815442</v>
+      </c>
+      <c r="F15" s="0">
+        <v>-0.019926155224890791</v>
+      </c>
+      <c r="G15" s="0">
+        <v>-0.017453292519425949</v>
+      </c>
+      <c r="H15" s="0">
+        <v>-0.014980429813961107</v>
+      </c>
+      <c r="I15" s="0">
+        <v>-0.01260676452015469</v>
+      </c>
+      <c r="J15" s="0">
+        <v>-0.0057788673842583691</v>
+      </c>
+      <c r="K15" s="0">
+        <v>0.0010490297516379515</v>
+      </c>
+      <c r="L15" s="0">
+        <v>0.66530948983677252</v>
+      </c>
+      <c r="M15" s="0">
+        <v>0.72644656961671272</v>
+      </c>
+      <c r="N15" s="0">
+        <v>0.78758364939665293</v>
+      </c>
+      <c r="O15" s="0">
+        <v>-0.056143140072090758</v>
+      </c>
+      <c r="P15" s="0">
+        <v>-0.048635072109916085</v>
+      </c>
+      <c r="Q15" s="0">
+        <v>-0.041127004147741411</v>
+      </c>
+      <c r="R15" s="0">
+        <v>0.78771096690985054</v>
+      </c>
+      <c r="S15" s="0">
+        <v>0.79456774951277209</v>
+      </c>
+      <c r="T15" s="0">
+        <v>0.80142453211569365</v>
+      </c>
+      <c r="U15" s="0">
+        <v>0.0057149965748189467</v>
+      </c>
+      <c r="V15" s="0">
+        <v>0.010664065481723634</v>
+      </c>
+      <c r="W15" s="0">
+        <v>0.015613134388628321</v>
+      </c>
+      <c r="X15" s="0">
+        <v>4.0930209428220437</v>
+      </c>
+      <c r="Y15" s="0">
+        <v>5.258020501155233</v>
+      </c>
+      <c r="Z15" s="0">
+        <v>6.4230200594884224</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0"/>
+      <c r="B16" s="0"/>
+      <c r="C16" s="0"/>
+      <c r="D16" s="0"/>
+      <c r="E16" s="0"/>
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
+      <c r="K16" s="0"/>
+      <c r="L16" s="0"/>
+      <c r="M16" s="0"/>
+      <c r="N16" s="0"/>
+      <c r="O16" s="0"/>
+      <c r="P16" s="0"/>
+      <c r="Q16" s="0"/>
+      <c r="R16" s="0"/>
+      <c r="S16" s="0"/>
+      <c r="T16" s="0"/>
+      <c r="U16" s="0"/>
+      <c r="V16" s="0"/>
+      <c r="W16" s="0"/>
+      <c r="X16" s="0"/>
+      <c r="Y16" s="0"/>
+      <c r="Z16" s="0"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="0"/>
+      <c r="C17" s="0">
+        <v>0.0055373343970319859</v>
+      </c>
+      <c r="D17" s="0">
+        <v>0.010397692775527207</v>
+      </c>
+      <c r="E17" s="0">
+        <v>0.015258051154022427</v>
+      </c>
+      <c r="F17" s="0">
+        <v>0.0017169799533122943</v>
+      </c>
+      <c r="G17" s="0">
+        <v>0.0027609987260931571</v>
+      </c>
+      <c r="H17" s="0">
+        <v>0.0038050174988740202</v>
+      </c>
+      <c r="I17" s="0">
+        <v>-0.0040551419603008379</v>
+      </c>
+      <c r="J17" s="0">
+        <v>-0.0011378340706119268</v>
+      </c>
+      <c r="K17" s="0">
+        <v>0.0017794738190769824</v>
+      </c>
+      <c r="L17" s="0">
+        <v>0.69832728629568164</v>
+      </c>
+      <c r="M17" s="0">
+        <v>0.74760238700613557</v>
+      </c>
+      <c r="N17" s="0">
+        <v>0.79687748771658984</v>
+      </c>
+      <c r="O17" s="0">
+        <v>-0.017526215161147812</v>
+      </c>
+      <c r="P17" s="0">
+        <v>-0.012942012746269115</v>
+      </c>
+      <c r="Q17" s="0">
+        <v>-0.0083578103313904206</v>
+      </c>
+      <c r="R17" s="0">
+        <v>0.76385003921020111</v>
+      </c>
+      <c r="S17" s="0">
+        <v>0.77503611960066598</v>
+      </c>
+      <c r="T17" s="0">
+        <v>0.78622219999113086</v>
+      </c>
+      <c r="U17" s="0">
+        <v>0.0031235551837530307</v>
+      </c>
+      <c r="V17" s="0">
+        <v>0.0054267117321361857</v>
+      </c>
+      <c r="W17" s="0">
+        <v>0.007729868280519343</v>
+      </c>
+      <c r="X17" s="0">
+        <v>-0.5294552099418296</v>
+      </c>
+      <c r="Y17" s="0">
+        <v>0.091482455797930226</v>
+      </c>
+      <c r="Z17" s="0">
+        <v>0.71242012153768974</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" s="0"/>
+      <c r="C18" s="0">
+        <v>0.0079768484677627885</v>
+      </c>
+      <c r="D18" s="0">
+        <v>0.0065015674177380826</v>
+      </c>
+      <c r="E18" s="0">
+        <v>0.0060179921608553809</v>
+      </c>
+      <c r="F18" s="0">
+        <v>0.0086030940313560952</v>
+      </c>
+      <c r="G18" s="0">
+        <v>0.0087830728879895927</v>
+      </c>
+      <c r="H18" s="0">
+        <v>0.0090793521345831942</v>
+      </c>
+      <c r="I18" s="0">
+        <v>0.013944191670417588</v>
+      </c>
+      <c r="J18" s="0">
+        <v>0.012276795588028256</v>
+      </c>
+      <c r="K18" s="0">
+        <v>0.011491074165993053</v>
+      </c>
+      <c r="L18" s="0">
+        <v>0.11855344276150329</v>
+      </c>
+      <c r="M18" s="0">
+        <v>0.081186884086595579</v>
+      </c>
+      <c r="N18" s="0">
+        <v>0.078168323331155753</v>
+      </c>
+      <c r="O18" s="0">
+        <v>0.018258947869323514</v>
+      </c>
+      <c r="P18" s="0">
+        <v>0.020489494147016615</v>
+      </c>
+      <c r="Q18" s="0">
+        <v>0.02347924220381074</v>
+      </c>
+      <c r="R18" s="0">
+        <v>0.065870059695426128</v>
+      </c>
+      <c r="S18" s="0">
+        <v>0.069006229397747781</v>
+      </c>
+      <c r="T18" s="0">
+        <v>0.072866323296130436</v>
+      </c>
+      <c r="U18" s="0">
+        <v>0.0042937489597340457</v>
+      </c>
+      <c r="V18" s="0">
+        <v>0.0035907861796131112</v>
+      </c>
+      <c r="W18" s="0">
+        <v>0.0041295299334551559</v>
+      </c>
+      <c r="X18" s="0">
+        <v>4.5747043602061517</v>
+      </c>
+      <c r="Y18" s="0">
+        <v>4.4351757374015817</v>
+      </c>
+      <c r="Z18" s="0">
+        <v>4.4387303276849011</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0"/>
+      <c r="B19" s="0"/>
+      <c r="C19" s="0"/>
+      <c r="D19" s="0"/>
+      <c r="E19" s="0"/>
+      <c r="F19" s="0"/>
+      <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
+      <c r="I19" s="0"/>
+      <c r="J19" s="0"/>
+      <c r="K19" s="0"/>
+      <c r="L19" s="0"/>
+      <c r="M19" s="0"/>
+      <c r="N19" s="0"/>
+      <c r="O19" s="0"/>
+      <c r="P19" s="0"/>
+      <c r="Q19" s="0"/>
+      <c r="R19" s="0"/>
+      <c r="S19" s="0"/>
+      <c r="T19" s="0"/>
+      <c r="U19" s="0"/>
+      <c r="V19" s="0"/>
+      <c r="W19" s="0"/>
+      <c r="X19" s="0"/>
+      <c r="Y19" s="0"/>
+      <c r="Z19" s="0"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="0"/>
+      <c r="C20" s="0"/>
+      <c r="D20" s="0">
+        <v>0.017453292513164097</v>
+      </c>
+      <c r="E20" s="0">
+        <v>0.018673228145556019</v>
+      </c>
+      <c r="F20" s="0"/>
+      <c r="G20" s="0">
+        <v>-0.00057089804056733912</v>
+      </c>
+      <c r="H20" s="0">
+        <v>-0.00048290366678096098</v>
+      </c>
+      <c r="I20" s="0"/>
+      <c r="J20" s="0">
+        <v>-0.000568744645598793</v>
+      </c>
+      <c r="K20" s="0">
+        <v>-0.00048060412778311887</v>
+      </c>
+      <c r="L20" s="0"/>
+      <c r="M20" s="0">
+        <v>0.7710967609274898</v>
+      </c>
+      <c r="N20" s="0">
+        <v>0.77337183458901759</v>
+      </c>
+      <c r="O20" s="0"/>
+      <c r="P20" s="0">
+        <v>-0.020828066719061161</v>
+      </c>
+      <c r="Q20" s="0">
+        <v>-0.020544972825856166</v>
+      </c>
+      <c r="R20" s="0"/>
+      <c r="S20" s="0">
+        <v>0.76781532726080359</v>
+      </c>
+      <c r="T20" s="0">
+        <v>0.77073532993273475</v>
+      </c>
+      <c r="U20" s="0"/>
+      <c r="V20" s="0">
+        <v>0.0048761525870936505</v>
+      </c>
+      <c r="W20" s="0">
+        <v>0.0051028436270321165</v>
+      </c>
+      <c r="X20" s="0"/>
+      <c r="Y20" s="0">
+        <v>-0.4746453244966028</v>
+      </c>
+      <c r="Z20" s="0">
+        <v>-0.46892554964112815</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="0"/>
+      <c r="C21" s="0">
+        <v>0.0056898040264526609</v>
+      </c>
+      <c r="D21" s="0">
+        <v>0.010583544209635899</v>
+      </c>
+      <c r="E21" s="0">
+        <v>0.014915411036279283</v>
+      </c>
+      <c r="F21" s="0">
+        <v>0.002147362083190032</v>
+      </c>
+      <c r="G21" s="0">
+        <v>0.0029192444552246827</v>
+      </c>
+      <c r="H21" s="0">
+        <v>0.003863041820641914</v>
+      </c>
+      <c r="I21" s="0">
+        <v>-0.0029301836083809362</v>
+      </c>
+      <c r="J21" s="0">
+        <v>-0.00031526235980879047</v>
+      </c>
+      <c r="K21" s="0">
+        <v>0.0022177986661390983</v>
+      </c>
+      <c r="L21" s="0">
+        <v>0.66209142107479546</v>
+      </c>
+      <c r="M21" s="0">
+        <v>0.70978349706506583</v>
+      </c>
+      <c r="N21" s="0">
+        <v>0.75321779256876586</v>
+      </c>
+      <c r="O21" s="0">
+        <v>-0.015289642471743352</v>
+      </c>
+      <c r="P21" s="0">
+        <v>-0.011439339045063602</v>
+      </c>
+      <c r="Q21" s="0">
+        <v>-0.0072019344466412796</v>
+      </c>
+      <c r="R21" s="0">
+        <v>0.72022629049052767</v>
+      </c>
+      <c r="S21" s="0">
+        <v>0.73308019709814942</v>
+      </c>
+      <c r="T21" s="0">
+        <v>0.74334909724093112</v>
+      </c>
+      <c r="U21" s="0">
+        <v>0.0031966922947518446</v>
+      </c>
+      <c r="V21" s="0">
+        <v>0.0052863302793382085</v>
+      </c>
+      <c r="W21" s="0">
+        <v>0.0073635528098986713</v>
+      </c>
+      <c r="X21" s="0">
+        <v>-0.21044523680758076</v>
+      </c>
+      <c r="Y21" s="0">
+        <v>0.31369219116905484</v>
+      </c>
+      <c r="Z21" s="0">
+        <v>0.86212391771230113</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="0"/>
-      <c r="C15" s="0">
-        <v>0.0061075251489893382</v>
-      </c>
-      <c r="D15" s="0">
-        <v>0.0067707825870930473</v>
-      </c>
-      <c r="E15" s="0">
-        <v>0.007478139325589603</v>
-      </c>
-      <c r="F15" s="0">
-        <v>0.0061075251685368788</v>
-      </c>
-      <c r="G15" s="0">
-        <v>0.0067707825870930612</v>
-      </c>
-      <c r="H15" s="0">
-        <v>0.0074781393046077036</v>
-      </c>
-      <c r="I15" s="0">
-        <v>0.070407391019634738</v>
-      </c>
-      <c r="J15" s="0">
-        <v>0.07735057216909072</v>
-      </c>
-      <c r="K15" s="0">
-        <v>0.09741737242325188</v>
-      </c>
-      <c r="L15" s="0">
-        <v>0.011678657499867719</v>
-      </c>
-      <c r="M15" s="0">
-        <v>0.013264739717743229</v>
-      </c>
-      <c r="N15" s="0">
-        <v>0.015263556338967362</v>
-      </c>
-      <c r="O15" s="0">
-        <v>0.036515361224403936</v>
-      </c>
-      <c r="P15" s="0">
-        <v>0.038562063483869202</v>
-      </c>
-      <c r="Q15" s="0">
-        <v>0.040670764168904784</v>
-      </c>
-      <c r="R15" s="0">
-        <v>0.00094704610194586223</v>
-      </c>
-      <c r="S15" s="0">
-        <v>0.001520124368323937</v>
-      </c>
-      <c r="T15" s="0">
-        <v>0.0021710308906964285</v>
-      </c>
-      <c r="U15" s="0">
-        <v>0.01105096546953771</v>
-      </c>
-      <c r="V15" s="0">
-        <v>0.010650316285598685</v>
-      </c>
-      <c r="W15" s="0">
-        <v>0.011360477405569018</v>
-      </c>
-      <c r="X15" s="0">
-        <v>0.31622776601683794</v>
-      </c>
-      <c r="Y15" s="0">
-        <v>0.31622776601683794</v>
-      </c>
-      <c r="Z15" s="0">
-        <v>0.31622776601683794</v>
+      <c r="B22" s="0"/>
+      <c r="C22" s="0">
+        <v>0.0074510434450682003</v>
+      </c>
+      <c r="D22" s="0">
+        <v>0.0061941959383005245</v>
+      </c>
+      <c r="E22" s="0">
+        <v>0.0059469386623042589</v>
+      </c>
+      <c r="F22" s="0">
+        <v>0.0081919751648099979</v>
+      </c>
+      <c r="G22" s="0">
+        <v>0.0081001234782882049</v>
+      </c>
+      <c r="H22" s="0">
+        <v>0.0083583711600579529</v>
+      </c>
+      <c r="I22" s="0">
+        <v>0.013739126046660813</v>
+      </c>
+      <c r="J22" s="0">
+        <v>0.011532914226126591</v>
+      </c>
+      <c r="K22" s="0">
+        <v>0.010644068646305755</v>
+      </c>
+      <c r="L22" s="0">
+        <v>0.18217995628340675</v>
+      </c>
+      <c r="M22" s="0">
+        <v>0.1778401804709539</v>
+      </c>
+      <c r="N22" s="0">
+        <v>0.18777051054328931</v>
+      </c>
+      <c r="O22" s="0">
+        <v>0.019208680467657207</v>
+      </c>
+      <c r="P22" s="0">
+        <v>0.020308743245423814</v>
+      </c>
+      <c r="Q22" s="0">
+        <v>0.022784293655124726</v>
+      </c>
+      <c r="R22" s="0">
+        <v>0.18495635350019876</v>
+      </c>
+      <c r="S22" s="0">
+        <v>0.18209019595113396</v>
+      </c>
+      <c r="T22" s="0">
+        <v>0.18488040288052651</v>
+      </c>
+      <c r="U22" s="0">
+        <v>0.0040079538467160045</v>
+      </c>
+      <c r="V22" s="0">
+        <v>0.003268767063605362</v>
+      </c>
+      <c r="W22" s="0">
+        <v>0.0038671027790681493</v>
+      </c>
+      <c r="X22" s="0">
+        <v>4.4458754435464991</v>
+      </c>
+      <c r="Y22" s="0">
+        <v>4.138756983074301</v>
+      </c>
+      <c r="Z22" s="0">
+        <v>4.1157489026912026</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" s="0"/>
+      <c r="C23" s="0">
+        <v>0.0057512927460635606</v>
+      </c>
+      <c r="D23" s="0">
+        <v>0.011000071011050957</v>
+      </c>
+      <c r="E23" s="0">
+        <v>0.015140582737144633</v>
+      </c>
+      <c r="F23" s="0">
+        <v>0.0021190649039728978</v>
+      </c>
+      <c r="G23" s="0">
+        <v>0.0026916362568016588</v>
+      </c>
+      <c r="H23" s="0">
+        <v>0.0035790447836771631</v>
+      </c>
+      <c r="I23" s="0">
+        <v>-0.0034714183932358146</v>
+      </c>
+      <c r="J23" s="0">
+        <v>-0.00086259607740874671</v>
+      </c>
+      <c r="K23" s="0">
+        <v>0.0014815442413058239</v>
+      </c>
+      <c r="L23" s="0">
+        <v>0.66323509156212346</v>
+      </c>
+      <c r="M23" s="0">
+        <v>0.71402391682962318</v>
+      </c>
+      <c r="N23" s="0">
+        <v>0.75502305664294067</v>
+      </c>
+      <c r="O23" s="0">
+        <v>-0.015401816394940046</v>
+      </c>
+      <c r="P23" s="0">
+        <v>-0.012080176781819277</v>
+      </c>
+      <c r="Q23" s="0">
+        <v>-0.0080842853739262269</v>
+      </c>
+      <c r="R23" s="0">
+        <v>0.7211459075457296</v>
+      </c>
+      <c r="S23" s="0">
+        <v>0.73578191643856139</v>
+      </c>
+      <c r="T23" s="0">
+        <v>0.74558774925866223</v>
+      </c>
+      <c r="U23" s="0">
+        <v>0.0034715426704498308</v>
+      </c>
+      <c r="V23" s="0">
+        <v>0.0055015710093655208</v>
+      </c>
+      <c r="W23" s="0">
+        <v>0.0074684289115522972</v>
+      </c>
+      <c r="X23" s="0">
+        <v>-3.859516388845726</v>
+      </c>
+      <c r="Y23" s="0">
+        <v>-3.2040004684085028</v>
+      </c>
+      <c r="Z23" s="0">
+        <v>-2.6974752947076008</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="0"/>
+      <c r="C24" s="0">
+        <v>0.0074265473982073858</v>
+      </c>
+      <c r="D24" s="0">
+        <v>0.0062674245166552791</v>
+      </c>
+      <c r="E24" s="0">
+        <v>0.0059425463997336281</v>
+      </c>
+      <c r="F24" s="0">
+        <v>0.0081633655159580529</v>
+      </c>
+      <c r="G24" s="0">
+        <v>0.0078861658866794891</v>
+      </c>
+      <c r="H24" s="0">
+        <v>0.0081661763964243315</v>
+      </c>
+      <c r="I24" s="0">
+        <v>0.013397431415092517</v>
+      </c>
+      <c r="J24" s="0">
+        <v>0.010643314860863463</v>
+      </c>
+      <c r="K24" s="0">
+        <v>0.0095162177082801364</v>
+      </c>
+      <c r="L24" s="0">
+        <v>0.18195703318612289</v>
+      </c>
+      <c r="M24" s="0">
+        <v>0.1732681114065103</v>
+      </c>
+      <c r="N24" s="0">
+        <v>0.18249435532637134</v>
+      </c>
+      <c r="O24" s="0">
+        <v>0.01909189478950965</v>
+      </c>
+      <c r="P24" s="0">
+        <v>0.019736922849756158</v>
+      </c>
+      <c r="Q24" s="0">
+        <v>0.022247504874922497</v>
+      </c>
+      <c r="R24" s="0">
+        <v>0.18520291741949305</v>
+      </c>
+      <c r="S24" s="0">
+        <v>0.17704928231926101</v>
+      </c>
+      <c r="T24" s="0">
+        <v>0.17968091338228692</v>
+      </c>
+      <c r="U24" s="0">
+        <v>0.0036686462521910131</v>
+      </c>
+      <c r="V24" s="0">
+        <v>0.0031241522829883166</v>
+      </c>
+      <c r="W24" s="0">
+        <v>0.0039582577617563227</v>
+      </c>
+      <c r="X24" s="0">
+        <v>5.2252889069125663</v>
+      </c>
+      <c r="Y24" s="0">
+        <v>4.798745697622433</v>
+      </c>
+      <c r="Z24" s="0">
+        <v>4.7414689766135148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>